<commit_message>
add logging nad fix empty rows in report
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -905,7 +905,11 @@
           <t>Мастер не указан</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -926,7 +930,11 @@
           <t>Сумма не является числом</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -947,7 +955,11 @@
           <t>Сумма не является числом</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -993,7 +1005,11 @@
           <t>Сумма не является числом</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1014,7 +1030,11 @@
           <t>Мастер не указан</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1060,7 +1080,11 @@
           <t>Сумма не является числом</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1081,7 +1105,11 @@
           <t>Сумма не является числом</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1127,7 +1155,11 @@
           <t>Мастер не указан</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1148,7 +1180,11 @@
           <t>Мастер не указан</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1169,7 +1205,11 @@
           <t>Мастер не указан</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1240,7 +1280,11 @@
           <t>Сумма не является числом</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1336,7 +1380,11 @@
           <t>Мастер не указан</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1407,7 +1455,11 @@
           <t>Мастер не указан</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1478,7 +1530,11 @@
           <t>Мастер не указан</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1499,7 +1555,11 @@
           <t>Мастер не указан</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1545,7 +1605,11 @@
           <t>Мастер не указан</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>значение отсутствует</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>